<commit_message>
Update P1 report files and Section4.2 timeslots
Update binary assets under 90007/P1: modify Section4.2_TimeSlots.xlsx, update the final report PDF, revise the pre-review DOCX backup, and add a PDF export of the pre-review backup for easier distribution.
</commit_message>
<xml_diff>
--- a/90007/P1/S4/4.2/Section4.2_TimeSlots.xlsx
+++ b/90007/P1/S4/4.2/Section4.2_TimeSlots.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\STUDY\IT_study_knowledge\90007\P1\S4\4.2\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06BE880F-F979-4661-9C05-CBC755831909}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="26860" windowHeight="12540" tabRatio="500" activeTab="1"/>
+    <workbookView xWindow="10704" yWindow="3636" windowWidth="24492" windowHeight="12444" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TimeSlots" sheetId="1" r:id="rId1"/>
@@ -153,14 +159,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="27">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -198,163 +198,13 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
+      <sz val="9"/>
+      <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="35">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -373,194 +223,8 @@
         <bgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="10">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -583,336 +247,173 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="41" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
   <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <dxfs count="17">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="1"/>
       </font>
       <border>
@@ -923,7 +424,7 @@
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="0"/>
       </font>
       <fill>
@@ -951,149 +452,32 @@
           <color theme="4"/>
         </bottom>
         <horizontal style="thin">
-          <color theme="4" tint="0.399975585192419"/>
+          <color theme="4" tint="0.39994506668294322"/>
         </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
       </border>
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
     <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
-      <tableStyleElement type="wholeTable" dxfId="6"/>
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="totalRow" dxfId="4"/>
-      <tableStyleElement type="firstColumn" dxfId="3"/>
-      <tableStyleElement type="lastColumn" dxfId="2"/>
-      <tableStyleElement type="firstRowStripe" dxfId="1"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
+      <tableStyleElement type="wholeTable" dxfId="16"/>
+      <tableStyleElement type="headerRow" dxfId="15"/>
+      <tableStyleElement type="totalRow" dxfId="14"/>
+      <tableStyleElement type="firstColumn" dxfId="13"/>
+      <tableStyleElement type="lastColumn" dxfId="12"/>
+      <tableStyleElement type="firstRowStripe" dxfId="11"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="10"/>
     </tableStyle>
     <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
-      <tableStyleElement type="headerRow" dxfId="16"/>
-      <tableStyleElement type="totalRow" dxfId="15"/>
-      <tableStyleElement type="firstRowStripe" dxfId="14"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
-      <tableStyleElement type="pageFieldValues" dxfId="7"/>
+      <tableStyleElement type="headerRow" dxfId="9"/>
+      <tableStyleElement type="totalRow" dxfId="8"/>
+      <tableStyleElement type="firstRowStripe" dxfId="7"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="6"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="5"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="4"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="3"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="2"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="1"/>
+      <tableStyleElement type="pageFieldValues" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -1168,12 +552,15 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="zh-CN"/>
   <c:roundedCorners val="0"/>
@@ -1204,7 +591,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr sz="1800" b="1" strike="noStrike">
+              <a:rPr lang="en-US" sz="1800" b="1" strike="noStrike">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
@@ -1213,17 +600,9 @@
               </a:rPr>
               <a:t>Bandwidth Across 4 Time Slots</a:t>
             </a:r>
-            <a:endParaRPr sz="1800" b="1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:uFillTx/>
-              <a:latin typeface="Calibri"/>
-            </a:endParaRPr>
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1299,6 +678,7 @@
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
                 </a:pPr>
+                <a:endParaRPr lang="zh-CN"/>
               </a:p>
             </c:txPr>
             <c:dLblPos val="r"/>
@@ -1311,9 +691,7 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
-                <c15:leaderLines/>
               </c:ext>
             </c:extLst>
           </c:dLbls>
@@ -1359,6 +737,11 @@
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-D61D-4DE9-B080-1AF3AF6B02C4}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
@@ -1420,6 +803,7 @@
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
                 </a:pPr>
+                <a:endParaRPr lang="zh-CN"/>
               </a:p>
             </c:txPr>
             <c:dLblPos val="r"/>
@@ -1432,9 +816,7 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
-                <c15:leaderLines/>
               </c:ext>
             </c:extLst>
           </c:dLbls>
@@ -1480,6 +862,11 @@
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-D61D-4DE9-B080-1AF3AF6B02C4}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
@@ -1528,7 +915,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr sz="1000" b="1" strike="noStrike">
+                  <a:rPr lang="en-US" sz="1000" b="1" strike="noStrike">
                     <a:solidFill>
                       <a:srgbClr val="000000"/>
                     </a:solidFill>
@@ -1537,17 +924,9 @@
                   </a:rPr>
                   <a:t>Time Slot</a:t>
                 </a:r>
-                <a:endParaRPr sz="1000" b="1" strike="noStrike">
-                  <a:solidFill>
-                    <a:srgbClr val="000000"/>
-                  </a:solidFill>
-                  <a:uFillTx/>
-                  <a:latin typeface="Calibri"/>
-                </a:endParaRPr>
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -1585,6 +964,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
+            <a:endParaRPr lang="zh-CN"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="28154084"/>
@@ -1630,7 +1010,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr sz="1000" b="1" strike="noStrike">
+                  <a:rPr lang="en-US" sz="1000" b="1" strike="noStrike">
                     <a:solidFill>
                       <a:srgbClr val="000000"/>
                     </a:solidFill>
@@ -1639,17 +1019,9 @@
                   </a:rPr>
                   <a:t>Bandwidth (Mbps)</a:t>
                 </a:r>
-                <a:endParaRPr sz="1000" b="1" strike="noStrike">
-                  <a:solidFill>
-                    <a:srgbClr val="000000"/>
-                  </a:solidFill>
-                  <a:uFillTx/>
-                  <a:latin typeface="Calibri"/>
-                </a:endParaRPr>
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -1687,6 +1059,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
+            <a:endParaRPr lang="zh-CN"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="2328475"/>
@@ -1696,7 +1069,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1720,6 +1092,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
+          <a:endParaRPr lang="zh-CN"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -1751,6 +1124,7 @@
       <a:pPr>
         <a:defRPr lang="zh-CN"/>
       </a:pPr>
+      <a:endParaRPr lang="zh-CN"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -1762,7 +1136,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>4</xdr:col>
@@ -1776,14 +1150,20 @@
       <xdr:row>19</xdr:row>
       <xdr:rowOff>170640</xdr:rowOff>
     </xdr:to>
-    <xdr:graphicFrame>
+    <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="5419725" y="190500"/>
-        <a:ext cx="7419340" cy="3804920"/>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1849,7 +1229,7 @@
         <a:cs typeface=""/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="">
+    <a:fmtScheme>
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1969,14 +1349,14 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K9"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
@@ -1989,7 +1369,7 @@
     <col min="11" max="11" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" spans="1:11">
+    <row r="1" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2024,7 +1404,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:11">
+    <row r="2" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>11</v>
       </c>
@@ -2057,7 +1437,7 @@
       </c>
       <c r="K2" s="5"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:11">
+    <row r="3" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>11</v>
       </c>
@@ -2086,11 +1466,11 @@
         <v>15</v>
       </c>
       <c r="J3" s="5">
-        <v>268.9</v>
+        <v>268.89999999999998</v>
       </c>
       <c r="K3" s="5"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:11">
+    <row r="4" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>11</v>
       </c>
@@ -2123,7 +1503,7 @@
       </c>
       <c r="K4" s="5"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:11">
+    <row r="5" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>11</v>
       </c>
@@ -2152,13 +1532,13 @@
         <v>15</v>
       </c>
       <c r="J5" s="5">
-        <v>304.4</v>
+        <v>301.8</v>
       </c>
       <c r="K5" s="5" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:11">
+    <row r="6" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>24</v>
       </c>
@@ -2191,7 +1571,7 @@
       </c>
       <c r="K6" s="5"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:11">
+    <row r="7" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>24</v>
       </c>
@@ -2220,11 +1600,11 @@
         <v>25</v>
       </c>
       <c r="J7" s="5">
-        <v>324.6</v>
+        <v>324.60000000000002</v>
       </c>
       <c r="K7" s="5"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:11">
+    <row r="8" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>24</v>
       </c>
@@ -2253,13 +1633,13 @@
         <v>25</v>
       </c>
       <c r="J8" s="5">
-        <v>326.1</v>
+        <v>326.10000000000002</v>
       </c>
       <c r="K8" s="5" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:11">
+    <row r="9" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>24</v>
       </c>
@@ -2288,30 +1668,29 @@
         <v>25</v>
       </c>
       <c r="J9" s="5">
-        <v>413.4</v>
+        <v>326.5</v>
       </c>
       <c r="K9" s="5" t="s">
         <v>32</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="16.8" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="3" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" spans="1:3">
+    <row r="1" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -2322,7 +1701,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:3">
+    <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -2333,7 +1712,7 @@
         <v>20.6</v>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:3">
+    <row r="3" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -2344,7 +1723,7 @@
         <v>22.2</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:3">
+    <row r="4" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -2355,7 +1734,7 @@
         <v>24.4</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:3">
+    <row r="5" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -2366,7 +1745,7 @@
         <v>20.8</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:3">
+    <row r="6" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>35</v>
       </c>
@@ -2379,20 +1758,20 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:3">
+    <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>36</v>
       </c>
       <c r="B7" s="4">
         <f>STDEV(B2:B5)</f>
-        <v>0.191485421551268</v>
+        <v>0.19148542155126799</v>
       </c>
       <c r="C7" s="4">
         <f>STDEV(C2:C5)</f>
         <v>1.75119007154183</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:3">
+    <row r="8" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>37</v>
       </c>
@@ -2405,7 +1784,7 @@
         <v>20.6</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:3">
+    <row r="9" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>38</v>
       </c>
@@ -2418,7 +1797,7 @@
         <v>24.4</v>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:3">
+    <row r="10" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>39</v>
       </c>
@@ -2432,9 +1811,9 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-  <headerFooter/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>